<commit_message>
fix: address investment import review findings
</commit_message>
<xml_diff>
--- a/samples/investments/zerodha-fictional.xlsx
+++ b/samples/investments/zerodha-fictional.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Client ID</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Equity - Example</t>
+  </si>
+  <si>
+    <t>MF</t>
   </si>
 </sst>
 </file>
@@ -509,7 +512,7 @@
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E9">
         <v>5</v>

</xml_diff>